<commit_message>
feat: adiciona modo verde (Green) com filtros Ano/Mês para Dashboard
</commit_message>
<xml_diff>
--- a/planilhas/Assistencia.xlsx
+++ b/planilhas/Assistencia.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Total de Chamados</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>Prioridade do Chamado</t>
+  </si>
+  <si>
+    <t>r4y</t>
   </si>
 </sst>
 </file>
@@ -117,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -126,6 +129,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,7 +424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="16384" width="12.5703125" style="3"/>
@@ -490,6 +494,59 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
     </row>
+    <row r="2" spans="1:26" ht="15.75" customHeight="1">
+      <c r="A2" s="3">
+        <v>23</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3">
+        <v>23</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3">
+        <v>4</v>
+      </c>
+      <c r="F2" s="3">
+        <v>5</v>
+      </c>
+      <c r="G2" s="3">
+        <v>6</v>
+      </c>
+      <c r="I2" s="3">
+        <v>899</v>
+      </c>
+      <c r="J2" s="3">
+        <v>54</v>
+      </c>
+      <c r="K2" s="3">
+        <v>3</v>
+      </c>
+      <c r="L2" s="3">
+        <v>88</v>
+      </c>
+      <c r="M2" s="3">
+        <v>65</v>
+      </c>
+      <c r="N2" s="3">
+        <v>789</v>
+      </c>
+      <c r="O2" s="3">
+        <v>678</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>900</v>
+      </c>
+      <c r="R2" s="3">
+        <v>670</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>